<commit_message>
Fix Excel fórmulas (REF_MOJ I10 no J10) y chips cuarteles sin ha
- generar_oa_excel.py: REF_MOJ corregido de J10 (texto label) a I10 (valor 4500)
  → elimina todos los #¡VALOR! en Dosis/ha, Nec.Total y Vol.solución desglose
  · ws2 H2 ref mojamiento corregida: OA!I10
  · Vol. solución desglose: C*OA!$I$10 (era $J$10)
  · Cuarteles texto: "15, 16, 18, 19, 20 (5 cuarteles)" sin ha individual
- oa_plantilla_v5.html: chips cuarteles muestran solo número (sin · ha)
  eliminado resumen agrupado (redundante si se enumeran igual)
  sup-box: "5 cuarteles · Superficie total: 23,11 ha"
- OA_plantilla_v5.xlsx: regenerado con fórmulas corregidas

https://claude.ai/code/session_01AagNdfym9AMaT4JJT35j2J
</commit_message>
<xml_diff>
--- a/erp_oa/OA_plantilla_v5.xlsx
+++ b/erp_oa/OA_plantilla_v5.xlsx
@@ -324,11 +324,11 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -987,7 +987,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>15–16, 18–20  (5 cuarteles)</t>
+          <t>15, 16, 18, 19, 20  (5 cuarteles)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1006,12 +1006,12 @@
       <c r="I10" s="9" t="n">
         <v>4500</v>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Cap. Estanque (L)</t>
         </is>
       </c>
-      <c r="K10" s="9" t="n">
+      <c r="K10" s="10" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
         <v>300</v>
       </c>
       <c r="E14" s="16">
-        <f>IFERROR(D14*J10/100/1000,"—")</f>
+        <f>IFERROR(D14*I10/100/1000,"—")</f>
         <v/>
       </c>
       <c r="F14" s="16">
@@ -1145,7 +1145,7 @@
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(D14*J10*G10/100/1000,"—")</f>
+        <f>IFERROR(D14*I10*G10/100/1000,"—")</f>
         <v/>
       </c>
       <c r="H14" s="17" t="n">
@@ -1182,7 +1182,7 @@
         <v>1000</v>
       </c>
       <c r="E15" s="16">
-        <f>IFERROR(D15*J10/100/1000,"—")</f>
+        <f>IFERROR(D15*I10/100/1000,"—")</f>
         <v/>
       </c>
       <c r="F15" s="16">
@@ -1190,7 +1190,7 @@
         <v/>
       </c>
       <c r="G15" s="16">
-        <f>IFERROR(D15*J10*G10/100/1000,"—")</f>
+        <f>IFERROR(D15*I10*G10/100/1000,"—")</f>
         <v/>
       </c>
       <c r="H15" s="20" t="n">
@@ -1225,7 +1225,7 @@
         <v>50</v>
       </c>
       <c r="E16" s="16">
-        <f>IFERROR(D16*J10/100/1000,"—")</f>
+        <f>IFERROR(D16*I10/100/1000,"—")</f>
         <v/>
       </c>
       <c r="F16" s="16">
@@ -1233,7 +1233,7 @@
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(D16*J10*G10/100/1000,"—")</f>
+        <f>IFERROR(D16*I10*G10/100/1000,"—")</f>
         <v/>
       </c>
       <c r="H16" s="22" t="n">
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="H2" s="38">
-        <f>OA!J10</f>
+        <f>OA!I10</f>
         <v/>
       </c>
       <c r="I2" s="37" t="inlineStr">
@@ -1633,7 +1633,7 @@
         <v>3.79</v>
       </c>
       <c r="D5" s="46">
-        <f>C5*OA!$J$10</f>
+        <f>C5*OA!$I$10</f>
         <v/>
       </c>
       <c r="E5" s="46">
@@ -1668,7 +1668,7 @@
         <v>4.31</v>
       </c>
       <c r="D6" s="46">
-        <f>C6*OA!$J$10</f>
+        <f>C6*OA!$I$10</f>
         <v/>
       </c>
       <c r="E6" s="46">
@@ -1703,7 +1703,7 @@
         <v>4.73</v>
       </c>
       <c r="D7" s="46">
-        <f>C7*OA!$J$10</f>
+        <f>C7*OA!$I$10</f>
         <v/>
       </c>
       <c r="E7" s="46">
@@ -1738,7 +1738,7 @@
         <v>5.14</v>
       </c>
       <c r="D8" s="46">
-        <f>C8*OA!$J$10</f>
+        <f>C8*OA!$I$10</f>
         <v/>
       </c>
       <c r="E8" s="46">
@@ -1773,7 +1773,7 @@
         <v>5.14</v>
       </c>
       <c r="D9" s="46">
-        <f>C9*OA!$J$10</f>
+        <f>C9*OA!$I$10</f>
         <v/>
       </c>
       <c r="E9" s="46">

</xml_diff>